<commit_message>
Updated NZL model - 2025-09-08 00:29
</commit_message>
<xml_diff>
--- a/VerveStacks_NZL/SysSettings.xlsx
+++ b/VerveStacks_NZL/SysSettings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_NZL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF06CC15-B1A6-44B9-8B4B-5F817D87BC15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D72A1C0-EE3B-4C0B-B780-E8ECC9D3E09E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="564" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="221">
   <si>
     <t>~BookRegions_Map</t>
   </si>
@@ -689,6 +689,12 @@
   </si>
   <si>
     <t>TWh</t>
+  </si>
+  <si>
+    <t>elc_wof-NZL</t>
+  </si>
+  <si>
+    <t>offshore wind electricity generation</t>
   </si>
   <si>
     <t>elc_won-NZL</t>
@@ -3254,6 +3260,24 @@
       <c r="E7" t="s">
         <v>18</v>
       </c>
+      <c r="M7" t="s">
+        <v>17</v>
+      </c>
+      <c r="N7" t="s">
+        <v>219</v>
+      </c>
+      <c r="O7" t="s">
+        <v>220</v>
+      </c>
+      <c r="P7" t="s">
+        <v>25</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>35</v>
+      </c>
+      <c r="R7" t="s">
+        <v>216</v>
+      </c>
     </row>
     <row r="8" spans="2:18">
       <c r="B8" t="s">

</xml_diff>